<commit_message>
test: Fix Integration test for attribution
</commit_message>
<xml_diff>
--- a/tests/integration/test_data/test_populate_attribution.xlsx
+++ b/tests/integration/test_data/test_populate_attribution.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Vidy/code/dnum/amendements-intelligents/tests/integration/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C347A2FE-FB82-704F-BC96-8DFE1A15427A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EC271D7-E81C-894E-B8D5-A97175BB4B8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="25600" windowHeight="28300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="125">
   <si>
     <t>amdt_idx</t>
   </si>
@@ -452,13 +452,6 @@
 - 1 expert : Marie Faugeron</t>
   </si>
   <si>
-    <t xml:space="preserve">I. – À la fin du I de l’article 1635 bis du code général des impôts, les mots : « et dans une limite annuelle égale à 7 500 € » sont supprimés.
-II. – Le code du service national est ainsi modifié :
-Le III de l’article L. 0121-2-1 est complété par un 9° ainsi rédigé :
-  « 9° Les composants de salaire établis mentionnés à l’article L. 0121-2-1 du présent code. » ;
-</t>
-  </si>
-  <si>
     <t>II. – La charge pour l’État et les collectivités territoriales est compensée par la création d’une taxe additionnelle à l’accise sur les tabacs prévue au chapitre IV du titre Ier du livre III du code des impositions sur les biens et services.</t>
   </si>
   <si>
@@ -469,13 +462,33 @@
 - 1 expert </t>
   </si>
   <si>
-    <t xml:space="preserve">  « 9° Les composantes salariales établis par un organisme de protection sociale mentionnés à l’article L. 0121-2-1 du présent code. » ;</t>
-  </si>
-  <si>
     <t>- 2 codes : Le code général des impôts, le code du service national 
 - 2 experts : Julien Dauce, Nathan Soto
 - 3 mot-clés : composants de salaire, organisme de protection sociale, composantes salariales
 - 2 experts : Julien Dauce, Nathan Soto</t>
+  </si>
+  <si>
+    <t>Rien ici</t>
+  </si>
+  <si>
+    <t>un organisme de protection sociale pour Nathan</t>
+  </si>
+  <si>
+    <t>- 1 mot-clé : organisme de protection sociale
+- 1 expert : Nathan Soto</t>
+  </si>
+  <si>
+    <t>I. – À la fin du I de l’article 1635 bis du code général des impôts, les mots : « et dans une limite annuelle égale à 7 500 € » sont supprimés.
+II. – Le code du service national est ainsi modifié :
+Le III de l’article L. 121-2-1 est complété par un 9° ainsi rédigé :
+  « 9° Les composants de salaire établis par un organisme de protection sociale mentionnés à l’article L. 0121-2-1 du présent code. » ;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I. – À la fin du I de l’article 1635 bis du code général des impôts, les mots : « et dans une limite annuelle égale à 7 500 € » sont supprimés.
+II. – Le code du service national est ainsi modifié :
+Le III de l’article L. 121-2-1 est complété par un 9° ainsi rédigé :
+  « 9° Les composants de salaire établis mentionnés à l’article L. 0121-2-1 du présent code. » ;
+</t>
   </si>
 </sst>
 </file>
@@ -493,22 +506,26 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
       <sz val="11"/>
       <color theme="10"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -2150,10 +2167,10 @@
         <v>104</v>
       </c>
       <c r="D44" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="E44" s="4" t="s">
         <v>117</v>
-      </c>
-      <c r="E44" s="4" t="s">
-        <v>118</v>
       </c>
       <c r="F44" s="7" t="s">
         <v>11</v>
@@ -2162,7 +2179,7 @@
         <v>12</v>
       </c>
       <c r="H44" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="144" x14ac:dyDescent="0.2">
@@ -2176,29 +2193,46 @@
         <v>101</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>102</v>
+        <v>123</v>
       </c>
       <c r="E45" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G45" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="H45" s="5" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="A46" s="3">
+        <v>45</v>
+      </c>
+      <c r="B46" s="3">
+        <v>44</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="D46" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="F45" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G45" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="H45" s="5" t="s">
+      <c r="E46" s="4" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B46" s="4"/>
-      <c r="C46" s="4"/>
-      <c r="D46" s="4"/>
-      <c r="E46" s="4"/>
-      <c r="F46" s="4"/>
-      <c r="G46" s="5"/>
-      <c r="H46" s="5"/>
+      <c r="F46" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G46" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="H46" s="5" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B47" s="4"/>

</xml_diff>